<commit_message>
San Fernando: Entorno Urbano REAL (NDVI + censo arboreo) + recalculo ITT
- Apunta PATHS a NDVI real (4 rasters 2023-2026) y censo arboreo filtrado (14329 arboles vivos)
- NDVI medio 0.179/0.216/0.212/0.217; score EntornoU 48.2/64.0/62.5/64.4 (antes 26.4 placeholder)
- ITT recalculado: 2023=46.9, 2024=57.1, 2025=54.3 (Consolidacion), 2026=78.4 (Transformacion)
- Excel actualizado (hoja Entorno_Urbano con NDVI/arbolado/habitabilidad reales)
- Ignora zips crudos de EarthEngine/shape ya extraidos
</commit_message>
<xml_diff>
--- a/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
+++ b/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
@@ -511,13 +511,13 @@
         <v>68.37</v>
       </c>
       <c r="E2" t="n">
-        <v>26.35</v>
+        <v>48.21</v>
       </c>
       <c r="F2" t="n">
         <v>54.91</v>
       </c>
       <c r="G2" t="n">
-        <v>43.21</v>
+        <v>46.93</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -544,13 +544,13 @@
         <v>69.93000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>26.35</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="F3" t="n">
         <v>58.13</v>
       </c>
       <c r="G3" t="n">
-        <v>50.7</v>
+        <v>57.1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -577,13 +577,13 @@
         <v>38.9</v>
       </c>
       <c r="E4" t="n">
-        <v>26.35</v>
+        <v>62.54</v>
       </c>
       <c r="F4" t="n">
         <v>64.36</v>
       </c>
       <c r="G4" t="n">
-        <v>48.12</v>
+        <v>54.27</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -610,13 +610,13 @@
         <v>64.63</v>
       </c>
       <c r="E5" t="n">
-        <v>26.35</v>
+        <v>64.39</v>
       </c>
       <c r="F5" t="n">
         <v>65.34</v>
       </c>
       <c r="G5" t="n">
-        <v>71.94</v>
+        <v>78.41</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -2444,19 +2444,23 @@
       <c r="A2" t="n">
         <v>2023</v>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>0.1787</v>
+      </c>
       <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>14329</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.2753</v>
+      </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>66.6651</v>
       </c>
       <c r="F2" t="n">
         <v>52.7</v>
       </c>
       <c r="G2" t="n">
-        <v>26.35</v>
+        <v>48.2135</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2473,19 +2477,23 @@
       <c r="A3" t="n">
         <v>2024</v>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>0.2157</v>
+      </c>
       <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>14329</v>
+      </c>
+      <c r="D3" t="n">
+        <v>72.6712</v>
+      </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>66.6651</v>
       </c>
       <c r="F3" t="n">
         <v>52.7</v>
       </c>
       <c r="G3" t="n">
-        <v>26.35</v>
+        <v>64.0121</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -2502,19 +2510,23 @@
       <c r="A4" t="n">
         <v>2025</v>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="n">
+        <v>0.2122</v>
+      </c>
       <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>14329</v>
+      </c>
+      <c r="D4" t="n">
+        <v>68.2632</v>
+      </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>66.6651</v>
       </c>
       <c r="F4" t="n">
         <v>52.7</v>
       </c>
       <c r="G4" t="n">
-        <v>26.35</v>
+        <v>62.5428</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -2531,19 +2543,23 @@
       <c r="A5" t="n">
         <v>2026</v>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="n">
+        <v>0.2166</v>
+      </c>
       <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>14329</v>
+      </c>
+      <c r="D5" t="n">
+        <v>73.7928</v>
+      </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>66.6651</v>
       </c>
       <c r="F5" t="n">
         <v>52.7</v>
       </c>
       <c r="G5" t="n">
-        <v>26.35</v>
+        <v>64.386</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
San Fernando: empleo (PERSONAL_OCUPADO) en DE + grafico comparacion subzonas
- DE pasa a 4 componentes: agrega empleo (33550/34846/35074/34969 personas por año,
  stock activo). Fuente PERSONAL_OCUPADO del registro_mercantil_2025_con_coordenadas.xlsx,
  preprocesado al consolidado con add_empleo_de_san_fernando.py (2992/4591 negocios)
- score_DE: 62.0/65.2/70.0/70.7 | ITT: 48.0/58.2/55.1/79.2
- Agrega grafico de la comparacion por subzonas (densidad por ha + conteos apilados)
</commit_message>
<xml_diff>
--- a/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
+++ b/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
@@ -514,10 +514,10 @@
         <v>48.21</v>
       </c>
       <c r="F2" t="n">
-        <v>54.91</v>
+        <v>61.98</v>
       </c>
       <c r="G2" t="n">
-        <v>46.93</v>
+        <v>47.99</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -547,10 +547,10 @@
         <v>64.01000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>58.13</v>
+        <v>65.19</v>
       </c>
       <c r="G3" t="n">
-        <v>57.1</v>
+        <v>58.16</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -580,10 +580,10 @@
         <v>62.54</v>
       </c>
       <c r="F4" t="n">
-        <v>64.36</v>
+        <v>70.01000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>54.27</v>
+        <v>55.12</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -613,10 +613,10 @@
         <v>64.39</v>
       </c>
       <c r="F5" t="n">
-        <v>65.34</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>78.41</v>
+        <v>79.20999999999999</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -3294,7 +3294,9 @@
       <c r="E2" t="n">
         <v>4029455479065</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>33550</v>
+      </c>
       <c r="G2" t="n">
         <v>29.52</v>
       </c>
@@ -3310,9 +3312,11 @@
       <c r="K2" t="n">
         <v>43.48</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>83.18000000000001</v>
+      </c>
       <c r="M2" t="n">
-        <v>54.91</v>
+        <v>61.98</v>
       </c>
     </row>
     <row r="3">
@@ -3333,7 +3337,9 @@
       <c r="E3" t="n">
         <v>4104047355269</v>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>34846</v>
+      </c>
       <c r="G3" t="n">
         <v>29.54</v>
       </c>
@@ -3349,9 +3355,11 @@
       <c r="K3" t="n">
         <v>44.86</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>86.39</v>
+      </c>
       <c r="M3" t="n">
-        <v>58.13</v>
+        <v>65.19</v>
       </c>
     </row>
     <row r="4">
@@ -3372,7 +3380,9 @@
       <c r="E4" t="n">
         <v>4771959231158</v>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>35074</v>
+      </c>
       <c r="G4" t="n">
         <v>29.59</v>
       </c>
@@ -3388,9 +3398,11 @@
       <c r="K4" t="n">
         <v>56.15</v>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>86.95999999999999</v>
+      </c>
       <c r="M4" t="n">
-        <v>64.36</v>
+        <v>70.01000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -3411,7 +3423,9 @@
       <c r="E5" t="n">
         <v>4779203372542</v>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>34969</v>
+      </c>
       <c r="G5" t="n">
         <v>29.59</v>
       </c>
@@ -3427,9 +3441,11 @@
       <c r="K5" t="n">
         <v>56.26</v>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>86.7</v>
+      </c>
       <c r="M5" t="n">
-        <v>65.34</v>
+        <v>70.68000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
San Fernando DE: desglose por sector social (Salud/Educacion/Deporte) + grafico y hoja Excel
- Clasifica empresas por CIIU (del registro mercantil 2025): Salud (86-88), Educacion (85),
  Deporte y recreacion (93 + ense. deportiva). Preprocesado add_sectores_de_san_fernando.py
- Celda DE-Sectores: empresas y empleo por sector/año (stock activo) + grafico (empresas barras,
  empleo lineas). Salud 372->451 (+21.2%, ~9000 empleos); Educacion 63->69; Deporte 16->20 (+25%)
- Excel: nueva hoja DE_Sectores_Salud_Dep_Edu; se quita hoja Auditoria_Spatial_Join (no necesaria)
- Sitio Pages SF: agrega grafico y tabla de sectores
</commit_message>
<xml_diff>
--- a/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
+++ b/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
@@ -16,9 +16,9 @@
     <sheet name="Vivienda_SecVivienda" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Vivienda_Resumen" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Desarrollo_Economico" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Indicadores_Trimestrales" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Comparacion_Subzonas" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Auditoria_Spatial_Join" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DE_Sectores_Salud_Dep_Edu" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Indicadores_Trimestrales" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Comparacion_Subzonas" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -640,6 +640,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>empresas_2023</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>empresas_2024</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>empresas_2025</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>empresas_2026</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>crecimiento_empresas_%</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>empleo_2023</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>empleo_2025</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>empleo_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Deporte y recreación</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H2" t="n">
+        <v>21</v>
+      </c>
+      <c r="I2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>63</v>
+      </c>
+      <c r="C3" t="n">
+        <v>67</v>
+      </c>
+      <c r="D3" t="n">
+        <v>71</v>
+      </c>
+      <c r="E3" t="n">
+        <v>69</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>198</v>
+      </c>
+      <c r="H3" t="n">
+        <v>203</v>
+      </c>
+      <c r="I3" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>372</v>
+      </c>
+      <c r="C4" t="n">
+        <v>415</v>
+      </c>
+      <c r="D4" t="n">
+        <v>459</v>
+      </c>
+      <c r="E4" t="n">
+        <v>451</v>
+      </c>
+      <c r="F4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8877</v>
+      </c>
+      <c r="H4" t="n">
+        <v>9013</v>
+      </c>
+      <c r="I4" t="n">
+        <v>9002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1288,7 +1453,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1550,132 +1715,6 @@
       </c>
       <c r="K6" t="n">
         <v>12.4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>fuente</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>metodo_espacial</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Homicidios</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>sjoin within al polígono</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hurtos</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>sjoin within al polígono</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Comparendos</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>sjoin within al polígono</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>VIF</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>sjoin within al polígono</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Siniestros</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>sjoin within al polígono</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Desarrollo Económico</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>sjoin within (Cámara geocodificada)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Vivienda (SISBÉN)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>sjoin + prorrateo por área (shapefile SISBÉN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Educación (Liceo Dptal)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sjoin de sedes al polígono (DANE 176001001745)</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
San Fernando DE-Sectores: agrega ingresos por sector (Salud/Educacion/Deporte)
- Suma ingresos operacionales del stock activo por sector y año + crecimiento vs 2023
- Grafico pasa a 3 paneles: empresas (barras), empleo (lineas), ingresos (lineas, escala log)
- Excel hoja DE_Sectores: columnas ingresos_2023/2025/2026 + crecimiento_ingresos_%
- Salud ~2.02 billones (+23%), Educacion ~12.7 mil mill (-6%), Deporte ~346 mill (+2%)
</commit_message>
<xml_diff>
--- a/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
+++ b/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
@@ -640,18 +640,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,37 +668,42 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>empresas_2024</t>
+          <t>empresas_2026</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>empresas_2025</t>
+          <t>crecimiento_empresas_%</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>empresas_2026</t>
+          <t>empleo_2023</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>crecimiento_empresas_%</t>
+          <t>empleo_2026</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>empleo_2023</t>
+          <t>ingresos_2023</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>empleo_2025</t>
+          <t>ingresos_2025</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>empleo_2026</t>
+          <t>ingresos_2026</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>crecimiento_ingresos_%</t>
         </is>
       </c>
     </row>
@@ -711,25 +717,28 @@
         <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F2" t="n">
         <v>20</v>
       </c>
-      <c r="F2" t="n">
-        <v>25</v>
-      </c>
       <c r="G2" t="n">
-        <v>18</v>
+        <v>340691681</v>
       </c>
       <c r="H2" t="n">
-        <v>21</v>
+        <v>345691681</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>345691681</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="3">
@@ -742,25 +751,28 @@
         <v>63</v>
       </c>
       <c r="C3" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D3" t="n">
-        <v>71</v>
+        <v>9.5</v>
       </c>
       <c r="E3" t="n">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="F3" t="n">
-        <v>9.5</v>
+        <v>199</v>
       </c>
       <c r="G3" t="n">
-        <v>198</v>
+        <v>13464016318</v>
       </c>
       <c r="H3" t="n">
-        <v>203</v>
+        <v>13464016318</v>
       </c>
       <c r="I3" t="n">
-        <v>199</v>
+        <v>12693710318</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-5.7</v>
       </c>
     </row>
     <row r="4">
@@ -773,25 +785,28 @@
         <v>372</v>
       </c>
       <c r="C4" t="n">
-        <v>415</v>
+        <v>451</v>
       </c>
       <c r="D4" t="n">
-        <v>459</v>
+        <v>21.2</v>
       </c>
       <c r="E4" t="n">
-        <v>451</v>
+        <v>8877</v>
       </c>
       <c r="F4" t="n">
-        <v>21.2</v>
+        <v>9002</v>
       </c>
       <c r="G4" t="n">
-        <v>8877</v>
+        <v>1651317119427</v>
       </c>
       <c r="H4" t="n">
-        <v>9013</v>
+        <v>2024384695875</v>
       </c>
       <c r="I4" t="n">
-        <v>9002</v>
+        <v>2024384695875</v>
+      </c>
+      <c r="J4" t="n">
+        <v>22.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
San Fernando DE-Sectores: ingresos como CORTE UNICO (no serie por anio)
- Los ingresos del registro mercantil son 1 valor por negocio (sin cronologia); armar serie
  por anio daba valores repetidos enganosos. Ahora 1 solo valor de ingresos por sector (stock
  activo 2026) + columna empresas_con_ingreso. Mismo criterio que habitabilidad de vivienda.
- Empresas y empleo siguen como serie por anio (si varian). Grafico: ingresos en barras por
  sector (no lineas temporales planas).
- Excel hoja DE_Sectores: quita columnas ingresos por anio, deja ingresos_operacionales unico
</commit_message>
<xml_diff>
--- a/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
+++ b/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -649,10 +649,8 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -688,22 +686,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ingresos_2023</t>
+          <t>empresas_con_ingreso</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>ingresos_2025</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>ingresos_2026</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>crecimiento_ingresos_%</t>
+          <t>ingresos_operacionales</t>
         </is>
       </c>
     </row>
@@ -729,17 +717,11 @@
         <v>20</v>
       </c>
       <c r="G2" t="n">
-        <v>340691681</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
         <v>345691681</v>
       </c>
-      <c r="I2" t="n">
-        <v>345691681</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1.5</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -763,16 +745,10 @@
         <v>199</v>
       </c>
       <c r="G3" t="n">
-        <v>13464016318</v>
+        <v>26</v>
       </c>
       <c r="H3" t="n">
-        <v>13464016318</v>
-      </c>
-      <c r="I3" t="n">
         <v>12693710318</v>
-      </c>
-      <c r="J3" t="n">
-        <v>-5.7</v>
       </c>
     </row>
     <row r="4">
@@ -797,16 +773,10 @@
         <v>9002</v>
       </c>
       <c r="G4" t="n">
-        <v>1651317119427</v>
+        <v>232</v>
       </c>
       <c r="H4" t="n">
         <v>2024384695875</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2024384695875</v>
-      </c>
-      <c r="J4" t="n">
-        <v>22.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
San Fernando DE-Sectores: Excel con empresas y empleo de los 4 anios (incluye 2024 y 2025)
- La hoja DE_Sectores solo traia empleo_2023 y empleo_2026; faltaban 2024 y 2025
- Ahora empresas_2023..2026 y empleo_2023..2026 completos + crecimiento_empleo_%
</commit_message>
<xml_diff>
--- a/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
+++ b/outputs/itt_corredor_san_fernando/ITT_Corredor_San_Fernando_Consolidado.xlsx
@@ -640,17 +640,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,30 +671,55 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>empresas_2024</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>empresas_2025</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>empresas_2026</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>crecimiento_empresas_%</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>empleo_2023</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>empleo_2024</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>empleo_2025</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>empleo_2026</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>crecimiento_empleo_%</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>empresas_con_ingreso</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ingresos_operacionales</t>
         </is>
@@ -705,21 +735,36 @@
         <v>16</v>
       </c>
       <c r="C2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E2" t="n">
         <v>20</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>25</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>18</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
+        <v>19</v>
+      </c>
+      <c r="I2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J2" t="n">
         <v>20</v>
       </c>
-      <c r="G2" t="n">
+      <c r="K2" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="L2" t="n">
         <v>5</v>
       </c>
-      <c r="H2" t="n">
+      <c r="M2" t="n">
         <v>345691681</v>
       </c>
     </row>
@@ -733,21 +778,36 @@
         <v>63</v>
       </c>
       <c r="C3" t="n">
+        <v>67</v>
+      </c>
+      <c r="D3" t="n">
+        <v>71</v>
+      </c>
+      <c r="E3" t="n">
         <v>69</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>9.5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>198</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
+        <v>200</v>
+      </c>
+      <c r="I3" t="n">
+        <v>203</v>
+      </c>
+      <c r="J3" t="n">
         <v>199</v>
       </c>
-      <c r="G3" t="n">
+      <c r="K3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L3" t="n">
         <v>26</v>
       </c>
-      <c r="H3" t="n">
+      <c r="M3" t="n">
         <v>12693710318</v>
       </c>
     </row>
@@ -761,21 +821,36 @@
         <v>372</v>
       </c>
       <c r="C4" t="n">
+        <v>415</v>
+      </c>
+      <c r="D4" t="n">
+        <v>459</v>
+      </c>
+      <c r="E4" t="n">
         <v>451</v>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>21.2</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>8877</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
+        <v>8959</v>
+      </c>
+      <c r="I4" t="n">
+        <v>9013</v>
+      </c>
+      <c r="J4" t="n">
         <v>9002</v>
       </c>
-      <c r="G4" t="n">
+      <c r="K4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L4" t="n">
         <v>232</v>
       </c>
-      <c r="H4" t="n">
+      <c r="M4" t="n">
         <v>2024384695875</v>
       </c>
     </row>

</xml_diff>